<commit_message>
feat: Enhance task finish functionality with package count and actual quantity calculations
</commit_message>
<xml_diff>
--- a/aspnet-core/prototype/领用配送接口FS(2).xlsx
+++ b/aspnet-core/prototype/领用配送接口FS(2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\module-zero-core-template\aspnet-core\prototype\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B18FB07-DF28-44D9-942E-3A9507D7F3B1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A799F0-0386-42F9-891D-2C477C15FE55}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目录" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="391">
   <si>
     <t>A-LM-ABAP-WMZC588</t>
   </si>
@@ -1268,6 +1268,114 @@
   </si>
   <si>
     <t>3,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>领料工厂</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>发料工厂</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>WERKS1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>WERKS2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BOLNR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHAR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>提单号</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>35,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>品种</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PZ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>10,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>在港箱量</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ZGXL</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XX</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>箱型</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>做箱日期</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>时间段</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>计划箱量</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>机台</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ZXRQ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SJD</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>JHXL</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>JT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>标准件重</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ZBZJZ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>QUAN</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>13,3</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1540,7 +1648,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1666,6 +1774,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1711,12 +1839,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2219,7 +2341,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="16.109375" style="14" customWidth="1"/>
@@ -2237,286 +2359,285 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="B4" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="15" t="s">
+    <row r="4" spans="1:8" s="48" customFormat="1">
+      <c r="B4" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="48" t="s">
         <v>56</v>
       </c>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="B5" s="15" t="s">
-        <v>290</v>
+      <c r="B5" s="7" t="s">
+        <v>365</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>291</v>
+        <v>367</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>165</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="B6" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>62</v>
+        <v>290</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>291</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="B7" s="15" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>67</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="B8" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="B9" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C9" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="15" t="s">
+      <c r="D9" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="15" customFormat="1">
-      <c r="B9" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="G9" s="60" t="s">
-        <v>309</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="15" customFormat="1">
       <c r="B10" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="G10" s="68" t="s">
+        <v>309</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="15" customFormat="1">
+      <c r="B11" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C11" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="7" t="s">
+      <c r="D11" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="G10" s="49"/>
-      <c r="H10" s="2" t="s">
+      <c r="G11" s="57"/>
+      <c r="H11" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
-      <c r="B11" s="7" t="s">
+    <row r="12" spans="1:8">
+      <c r="B12" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C12" s="7" t="s">
         <v>311</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D12" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="2" t="s">
+      <c r="G12" s="56"/>
+      <c r="H12" s="2" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
-      <c r="B12" s="15" t="s">
+    <row r="13" spans="1:8">
+      <c r="B13" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C13" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D13" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E13" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="48"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" s="15" customFormat="1">
-      <c r="B13" s="2" t="s">
+      <c r="G13" s="56"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" s="15" customFormat="1">
+      <c r="B14" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="54" t="s">
         <v>152</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="D14" s="54" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="49"/>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" s="2" customFormat="1">
-      <c r="B14" s="2" t="s">
+      <c r="G14" s="57"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1">
+      <c r="B15" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="B15" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>165</v>
-      </c>
+      <c r="G15" s="6"/>
     </row>
     <row r="16" spans="1:8">
       <c r="B16" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" s="7" t="s">
+      <c r="D17" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="B17" s="15" t="s">
+    <row r="18" spans="2:7">
+      <c r="B18" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C18" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E17" s="15" t="s">
+      <c r="D18" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="B18" s="7" t="s">
+    <row r="19" spans="2:7">
+      <c r="B19" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C19" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D19" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E19" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
-      <c r="B19" s="15" t="s">
+    <row r="20" spans="2:7">
+      <c r="B20" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C20" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="15" t="s">
+      <c r="D20" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
-      <c r="B20" s="15" t="s">
+    <row r="21" spans="2:7">
+      <c r="B21" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C21" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D21" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E21" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="2" customFormat="1">
-      <c r="B21" s="2" t="s">
+    <row r="22" spans="2:7" s="2" customFormat="1">
+      <c r="B22" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" s="2" customFormat="1">
-      <c r="B22" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>55</v>
@@ -2524,94 +2645,228 @@
       <c r="E22" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="6"/>
-    </row>
-    <row r="23" spans="1:7" s="2" customFormat="1">
+      <c r="F22" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" s="2" customFormat="1">
       <c r="B23" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="2:7" s="2" customFormat="1">
+      <c r="B24" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="6"/>
-    </row>
-    <row r="24" spans="1:7" s="2" customFormat="1">
-      <c r="B24" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7" s="2" customFormat="1">
+    <row r="25" spans="2:7" s="2" customFormat="1">
+      <c r="B25" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>56</v>
+      </c>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" s="15" customFormat="1"/>
-    <row r="27" spans="1:7">
-      <c r="A27" s="15" t="s">
+    <row r="26" spans="2:7" s="2" customFormat="1">
+      <c r="B26" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" spans="2:7" s="49" customFormat="1">
+      <c r="B27" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" spans="2:7" s="49" customFormat="1">
+      <c r="B28" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="2:7" s="49" customFormat="1">
+      <c r="B29" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="30" spans="2:7" s="49" customFormat="1">
+      <c r="B30" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" spans="2:7" s="49" customFormat="1">
+      <c r="B31" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" spans="2:7" s="49" customFormat="1">
+      <c r="B32" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="1:7" s="49" customFormat="1">
+      <c r="B33" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" spans="1:7" s="15" customFormat="1"/>
+    <row r="35" spans="1:7">
+      <c r="A35" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B35" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C35" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D35" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
-      <c r="B28" s="62" t="s">
+    <row r="36" spans="1:7">
+      <c r="B36" s="70" t="s">
         <v>123</v>
       </c>
-      <c r="C28" s="61" t="s">
+      <c r="C36" s="69" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="61" t="s">
+      <c r="D36" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="60" t="s">
+      <c r="E36" s="68" t="s">
         <v>317</v>
       </c>
-      <c r="F28" s="49"/>
-      <c r="G28" s="48"/>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="B29" s="48"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="15" t="s">
+      <c r="F36" s="57"/>
+      <c r="G36" s="56"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="B37" s="56"/>
+      <c r="C37" s="57"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="15" t="s">
         <v>126</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="G9:G13"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="G10:G14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2823,16 +3078,16 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="15" t="s">
@@ -3092,7 +3347,7 @@
       <c r="F23" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G23" s="50" t="s">
+      <c r="G23" s="58" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3112,7 +3367,7 @@
       <c r="F24" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G24" s="49"/>
+      <c r="G24" s="57"/>
     </row>
     <row r="25" spans="2:8">
       <c r="B25" s="15" t="s">
@@ -3130,7 +3385,7 @@
       <c r="F25" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G25" s="49"/>
+      <c r="G25" s="57"/>
     </row>
     <row r="26" spans="2:8">
       <c r="B26" s="15" t="s">
@@ -3148,7 +3403,7 @@
       <c r="F26" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G26" s="49"/>
+      <c r="G26" s="57"/>
     </row>
     <row r="27" spans="2:8" s="9" customFormat="1">
       <c r="B27" s="9" t="s">
@@ -3284,7 +3539,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="16.21875" style="14" customWidth="1"/>
@@ -3560,7 +3815,7 @@
       <c r="E22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="47" t="s">
+      <c r="F22" s="55" t="s">
         <v>153</v>
       </c>
     </row>
@@ -3577,7 +3832,7 @@
       <c r="E23" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="51"/>
+      <c r="F23" s="59"/>
     </row>
     <row r="24" spans="2:6" s="2" customFormat="1">
       <c r="B24" s="2" t="s">
@@ -3592,7 +3847,7 @@
       <c r="E24" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F24" s="51"/>
+      <c r="F24" s="59"/>
     </row>
     <row r="25" spans="2:6" s="2" customFormat="1">
       <c r="B25" s="2" t="s">
@@ -3607,7 +3862,7 @@
       <c r="E25" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="51"/>
+      <c r="F25" s="59"/>
     </row>
     <row r="26" spans="2:6" s="2" customFormat="1">
       <c r="B26" s="2" t="s">
@@ -3622,7 +3877,7 @@
       <c r="E26" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F26" s="51"/>
+      <c r="F26" s="59"/>
     </row>
     <row r="27" spans="2:6">
       <c r="B27" s="7" t="s">
@@ -3637,7 +3892,7 @@
       <c r="E27" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F27" s="48"/>
+      <c r="F27" s="56"/>
     </row>
     <row r="28" spans="2:6">
       <c r="B28" s="7" t="s">
@@ -3652,7 +3907,7 @@
       <c r="E28" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F28" s="48"/>
+      <c r="F28" s="56"/>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" s="15" t="s">
@@ -3667,7 +3922,7 @@
       <c r="E29" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="48"/>
+      <c r="F29" s="56"/>
     </row>
     <row r="30" spans="2:6">
       <c r="B30" s="15" t="s">
@@ -3682,7 +3937,7 @@
       <c r="E30" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="F30" s="48"/>
+      <c r="F30" s="56"/>
     </row>
     <row r="31" spans="2:6">
       <c r="B31" s="15" t="s">
@@ -3697,7 +3952,7 @@
       <c r="E31" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="48"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="2:6">
       <c r="F32" s="13"/>
@@ -3752,16 +4007,16 @@
       <c r="F36" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="G36" s="47" t="s">
+      <c r="G36" s="55" t="s">
         <v>184</v>
       </c>
-      <c r="H36" s="49"/>
-      <c r="I36" s="49"/>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
-      <c r="L36" s="49"/>
-      <c r="M36" s="49"/>
-      <c r="N36" s="49"/>
+      <c r="H36" s="57"/>
+      <c r="I36" s="57"/>
+      <c r="J36" s="57"/>
+      <c r="K36" s="57"/>
+      <c r="L36" s="57"/>
+      <c r="M36" s="57"/>
+      <c r="N36" s="57"/>
     </row>
     <row r="37" spans="2:14">
       <c r="B37" s="15" t="s">
@@ -3776,16 +4031,16 @@
       <c r="E37" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="G37" s="47" t="s">
+      <c r="G37" s="55" t="s">
         <v>188</v>
       </c>
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49"/>
-      <c r="M37" s="49"/>
-      <c r="N37" s="49"/>
+      <c r="H37" s="57"/>
+      <c r="I37" s="57"/>
+      <c r="J37" s="57"/>
+      <c r="K37" s="57"/>
+      <c r="L37" s="57"/>
+      <c r="M37" s="57"/>
+      <c r="N37" s="57"/>
     </row>
     <row r="38" spans="2:14" s="34" customFormat="1">
       <c r="B38" s="7" t="s">
@@ -3803,144 +4058,162 @@
       <c r="F38" s="33"/>
       <c r="G38" s="32"/>
     </row>
-    <row r="40" spans="2:14">
-      <c r="B40" s="15" t="s">
+    <row r="39" spans="2:14">
+      <c r="B39" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" s="53" customFormat="1">
+      <c r="B40" s="52"/>
+      <c r="F40" s="52"/>
+    </row>
+    <row r="41" spans="2:14">
+      <c r="B41" s="15" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="41" spans="2:14">
-      <c r="B41" s="52" t="s">
+    <row r="42" spans="2:14">
+      <c r="B42" s="60" t="s">
         <v>190</v>
       </c>
-      <c r="C41" s="49"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="49"/>
-      <c r="J41" s="49"/>
-      <c r="K41" s="49"/>
-      <c r="L41" s="49"/>
-      <c r="M41" s="49"/>
-    </row>
-    <row r="42" spans="2:14">
-      <c r="B42" s="48"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="49"/>
-      <c r="K42" s="49"/>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="57"/>
+      <c r="E42" s="57"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="57"/>
+      <c r="H42" s="57"/>
+      <c r="I42" s="57"/>
+      <c r="J42" s="57"/>
+      <c r="K42" s="57"/>
+      <c r="L42" s="57"/>
+      <c r="M42" s="57"/>
     </row>
     <row r="43" spans="2:14">
-      <c r="B43" s="48"/>
-      <c r="C43" s="49"/>
-      <c r="D43" s="49"/>
-      <c r="E43" s="49"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="49"/>
-      <c r="J43" s="49"/>
-      <c r="K43" s="49"/>
-      <c r="L43" s="49"/>
-      <c r="M43" s="49"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="57"/>
+      <c r="L43" s="57"/>
+      <c r="M43" s="57"/>
     </row>
     <row r="44" spans="2:14">
-      <c r="B44" s="48"/>
-      <c r="C44" s="49"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="49"/>
-      <c r="J44" s="49"/>
-      <c r="K44" s="49"/>
-      <c r="L44" s="49"/>
-      <c r="M44" s="49"/>
+      <c r="B44" s="56"/>
+      <c r="C44" s="57"/>
+      <c r="D44" s="57"/>
+      <c r="E44" s="57"/>
+      <c r="F44" s="56"/>
+      <c r="G44" s="57"/>
+      <c r="H44" s="57"/>
+      <c r="I44" s="57"/>
+      <c r="J44" s="57"/>
+      <c r="K44" s="57"/>
+      <c r="L44" s="57"/>
+      <c r="M44" s="57"/>
     </row>
     <row r="45" spans="2:14">
-      <c r="B45" s="48"/>
-      <c r="C45" s="49"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="49"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="49"/>
-      <c r="J45" s="49"/>
-      <c r="K45" s="49"/>
-      <c r="L45" s="49"/>
-      <c r="M45" s="49"/>
+      <c r="B45" s="56"/>
+      <c r="C45" s="57"/>
+      <c r="D45" s="57"/>
+      <c r="E45" s="57"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="57"/>
+      <c r="H45" s="57"/>
+      <c r="I45" s="57"/>
+      <c r="J45" s="57"/>
+      <c r="K45" s="57"/>
+      <c r="L45" s="57"/>
+      <c r="M45" s="57"/>
     </row>
     <row r="46" spans="2:14">
-      <c r="B46" s="48"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="49"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49"/>
-      <c r="I46" s="49"/>
-      <c r="J46" s="49"/>
-      <c r="K46" s="49"/>
-      <c r="L46" s="49"/>
-      <c r="M46" s="49"/>
+      <c r="B46" s="56"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="56"/>
+      <c r="G46" s="57"/>
+      <c r="H46" s="57"/>
+      <c r="I46" s="57"/>
+      <c r="J46" s="57"/>
+      <c r="K46" s="57"/>
+      <c r="L46" s="57"/>
+      <c r="M46" s="57"/>
     </row>
     <row r="47" spans="2:14">
-      <c r="B47" s="48"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="49"/>
-      <c r="I47" s="49"/>
-      <c r="J47" s="49"/>
-      <c r="K47" s="49"/>
-      <c r="L47" s="49"/>
-      <c r="M47" s="49"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="57"/>
+      <c r="E47" s="57"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="57"/>
+      <c r="K47" s="57"/>
+      <c r="L47" s="57"/>
+      <c r="M47" s="57"/>
     </row>
     <row r="48" spans="2:14">
-      <c r="B48" s="48"/>
-      <c r="C48" s="49"/>
-      <c r="D48" s="49"/>
-      <c r="E48" s="49"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="49"/>
-      <c r="I48" s="49"/>
-      <c r="J48" s="49"/>
-      <c r="K48" s="49"/>
-      <c r="L48" s="49"/>
-      <c r="M48" s="49"/>
+      <c r="B48" s="56"/>
+      <c r="C48" s="57"/>
+      <c r="D48" s="57"/>
+      <c r="E48" s="57"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="57"/>
+      <c r="H48" s="57"/>
+      <c r="I48" s="57"/>
+      <c r="J48" s="57"/>
+      <c r="K48" s="57"/>
+      <c r="L48" s="57"/>
+      <c r="M48" s="57"/>
     </row>
     <row r="49" spans="2:13">
-      <c r="B49" s="48"/>
-      <c r="C49" s="49"/>
-      <c r="D49" s="49"/>
-      <c r="E49" s="49"/>
-      <c r="F49" s="48"/>
-      <c r="G49" s="49"/>
-      <c r="H49" s="49"/>
-      <c r="I49" s="49"/>
-      <c r="J49" s="49"/>
-      <c r="K49" s="49"/>
-      <c r="L49" s="49"/>
-      <c r="M49" s="49"/>
+      <c r="B49" s="56"/>
+      <c r="C49" s="57"/>
+      <c r="D49" s="57"/>
+      <c r="E49" s="57"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="57"/>
+      <c r="H49" s="57"/>
+      <c r="I49" s="57"/>
+      <c r="J49" s="57"/>
+      <c r="K49" s="57"/>
+      <c r="L49" s="57"/>
+      <c r="M49" s="57"/>
+    </row>
+    <row r="50" spans="2:13">
+      <c r="B50" s="56"/>
+      <c r="C50" s="57"/>
+      <c r="D50" s="57"/>
+      <c r="E50" s="57"/>
+      <c r="F50" s="56"/>
+      <c r="G50" s="57"/>
+      <c r="H50" s="57"/>
+      <c r="I50" s="57"/>
+      <c r="J50" s="57"/>
+      <c r="K50" s="57"/>
+      <c r="L50" s="57"/>
+      <c r="M50" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="G37:N37"/>
     <mergeCell ref="F22:F31"/>
-    <mergeCell ref="B41:M49"/>
+    <mergeCell ref="B42:M50"/>
     <mergeCell ref="G36:N36"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -5021,13 +5294,13 @@
       <c r="E4" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="53" t="s">
+      <c r="F4" s="61" t="s">
         <v>347</v>
       </c>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
       <c r="K4" s="35"/>
       <c r="L4" s="35"/>
       <c r="M4" s="35"/>
@@ -5074,7 +5347,7 @@
       <c r="D6" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="50" t="s">
         <v>359</v>
       </c>
       <c r="F6" s="35" t="s">
@@ -5259,10 +5532,10 @@
       <c r="B13" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="64" t="s">
+      <c r="C13" s="51" t="s">
         <v>360</v>
       </c>
-      <c r="D13" s="64" t="s">
+      <c r="D13" s="51" t="s">
         <v>361</v>
       </c>
       <c r="E13" s="35" t="s">
@@ -5286,13 +5559,13 @@
       <c r="B14" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="C14" s="64" t="s">
+      <c r="C14" s="51" t="s">
         <v>362</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" s="50" t="s">
         <v>361</v>
       </c>
-      <c r="E14" s="64" t="s">
+      <c r="E14" s="51" t="s">
         <v>363</v>
       </c>
       <c r="F14" s="35"/>
@@ -5326,14 +5599,14 @@
       <c r="G15" s="35"/>
       <c r="H15" s="35"/>
       <c r="I15" s="35"/>
-      <c r="J15" s="52" t="s">
+      <c r="J15" s="60" t="s">
         <v>295</v>
       </c>
-      <c r="K15" s="58"/>
-      <c r="L15" s="58"/>
-      <c r="M15" s="58"/>
-      <c r="N15" s="58"/>
-      <c r="O15" s="58"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="66"/>
+      <c r="M15" s="66"/>
+      <c r="N15" s="66"/>
+      <c r="O15" s="66"/>
       <c r="P15" s="35"/>
       <c r="Q15" s="35"/>
     </row>
@@ -5355,12 +5628,12 @@
       <c r="G16" s="35"/>
       <c r="H16" s="35"/>
       <c r="I16" s="35"/>
-      <c r="J16" s="58"/>
-      <c r="K16" s="58"/>
-      <c r="L16" s="58"/>
-      <c r="M16" s="58"/>
-      <c r="N16" s="58"/>
-      <c r="O16" s="58"/>
+      <c r="J16" s="66"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="66"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="66"/>
+      <c r="O16" s="66"/>
       <c r="P16" s="35"/>
       <c r="Q16" s="35"/>
     </row>
@@ -5382,12 +5655,12 @@
       <c r="G17" s="35"/>
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
-      <c r="J17" s="58"/>
-      <c r="K17" s="58"/>
-      <c r="L17" s="58"/>
-      <c r="M17" s="58"/>
-      <c r="N17" s="58"/>
-      <c r="O17" s="58"/>
+      <c r="J17" s="66"/>
+      <c r="K17" s="66"/>
+      <c r="L17" s="66"/>
+      <c r="M17" s="66"/>
+      <c r="N17" s="66"/>
+      <c r="O17" s="66"/>
       <c r="P17" s="35"/>
       <c r="Q17" s="35"/>
     </row>
@@ -5409,12 +5682,12 @@
       <c r="G18" s="35"/>
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
-      <c r="J18" s="58"/>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="58"/>
-      <c r="N18" s="58"/>
-      <c r="O18" s="58"/>
+      <c r="J18" s="66"/>
+      <c r="K18" s="66"/>
+      <c r="L18" s="66"/>
+      <c r="M18" s="66"/>
+      <c r="N18" s="66"/>
+      <c r="O18" s="66"/>
       <c r="P18" s="35"/>
       <c r="Q18" s="35"/>
     </row>
@@ -5428,12 +5701,12 @@
       <c r="G19" s="35"/>
       <c r="H19" s="35"/>
       <c r="I19" s="35"/>
-      <c r="J19" s="58"/>
-      <c r="K19" s="58"/>
-      <c r="L19" s="58"/>
-      <c r="M19" s="58"/>
-      <c r="N19" s="58"/>
-      <c r="O19" s="58"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="66"/>
+      <c r="L19" s="66"/>
+      <c r="M19" s="66"/>
+      <c r="N19" s="66"/>
+      <c r="O19" s="66"/>
       <c r="P19" s="35"/>
       <c r="Q19" s="35"/>
     </row>
@@ -5447,12 +5720,12 @@
       <c r="G20" s="35"/>
       <c r="H20" s="35"/>
       <c r="I20" s="35"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="58"/>
-      <c r="N20" s="58"/>
-      <c r="O20" s="58"/>
+      <c r="J20" s="66"/>
+      <c r="K20" s="66"/>
+      <c r="L20" s="66"/>
+      <c r="M20" s="66"/>
+      <c r="N20" s="66"/>
+      <c r="O20" s="66"/>
       <c r="P20" s="35"/>
       <c r="Q20" s="35"/>
     </row>
@@ -5466,12 +5739,12 @@
       <c r="G21" s="35"/>
       <c r="H21" s="35"/>
       <c r="I21" s="35"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="58"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="58"/>
-      <c r="O21" s="58"/>
+      <c r="J21" s="66"/>
+      <c r="K21" s="66"/>
+      <c r="L21" s="66"/>
+      <c r="M21" s="66"/>
+      <c r="N21" s="66"/>
+      <c r="O21" s="66"/>
       <c r="P21" s="35"/>
       <c r="Q21" s="35"/>
     </row>
@@ -5495,47 +5768,47 @@
       <c r="G22" s="35"/>
       <c r="H22" s="35"/>
       <c r="I22" s="35"/>
-      <c r="J22" s="58"/>
-      <c r="K22" s="58"/>
-      <c r="L22" s="58"/>
-      <c r="M22" s="58"/>
-      <c r="N22" s="58"/>
-      <c r="O22" s="58"/>
+      <c r="J22" s="66"/>
+      <c r="K22" s="66"/>
+      <c r="L22" s="66"/>
+      <c r="M22" s="66"/>
+      <c r="N22" s="66"/>
+      <c r="O22" s="66"/>
       <c r="P22" s="35"/>
       <c r="Q22" s="35"/>
     </row>
     <row r="23" spans="1:17" ht="34.950000000000003" customHeight="1">
       <c r="A23" s="35"/>
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="64" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="56" t="s">
+      <c r="D23" s="64" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="57" t="s">
+      <c r="E23" s="65" t="s">
         <v>348</v>
       </c>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
       <c r="H23" s="35"/>
       <c r="I23" s="35"/>
-      <c r="J23" s="58"/>
-      <c r="K23" s="58"/>
-      <c r="L23" s="58"/>
-      <c r="M23" s="58"/>
-      <c r="N23" s="58"/>
-      <c r="O23" s="58"/>
+      <c r="J23" s="66"/>
+      <c r="K23" s="66"/>
+      <c r="L23" s="66"/>
+      <c r="M23" s="66"/>
+      <c r="N23" s="66"/>
+      <c r="O23" s="66"/>
       <c r="P23" s="35"/>
       <c r="Q23" s="35"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="35"/>
-      <c r="B24" s="55"/>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
+      <c r="B24" s="63"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
       <c r="E24" s="43" t="s">
         <v>126</v>
       </c>
@@ -5543,12 +5816,12 @@
       <c r="G24" s="44"/>
       <c r="H24" s="35"/>
       <c r="I24" s="35"/>
-      <c r="J24" s="58"/>
-      <c r="K24" s="58"/>
-      <c r="L24" s="58"/>
-      <c r="M24" s="58"/>
-      <c r="N24" s="58"/>
-      <c r="O24" s="58"/>
+      <c r="J24" s="66"/>
+      <c r="K24" s="66"/>
+      <c r="L24" s="66"/>
+      <c r="M24" s="66"/>
+      <c r="N24" s="66"/>
+      <c r="O24" s="66"/>
       <c r="P24" s="35"/>
       <c r="Q24" s="35"/>
     </row>
@@ -5597,12 +5870,12 @@
       <c r="G26" s="44"/>
       <c r="H26" s="35"/>
       <c r="I26" s="35"/>
-      <c r="J26" s="54" t="s">
+      <c r="J26" s="62" t="s">
         <v>349</v>
       </c>
-      <c r="K26" s="54"/>
-      <c r="L26" s="54"/>
-      <c r="M26" s="54"/>
+      <c r="K26" s="62"/>
+      <c r="L26" s="62"/>
+      <c r="M26" s="62"/>
       <c r="N26" s="35"/>
       <c r="O26" s="35"/>
       <c r="P26" s="35"/>
@@ -5626,10 +5899,10 @@
       <c r="G27" s="44"/>
       <c r="H27" s="35"/>
       <c r="I27" s="35"/>
-      <c r="J27" s="54"/>
-      <c r="K27" s="54"/>
-      <c r="L27" s="54"/>
-      <c r="M27" s="54"/>
+      <c r="J27" s="62"/>
+      <c r="K27" s="62"/>
+      <c r="L27" s="62"/>
+      <c r="M27" s="62"/>
       <c r="N27" s="35"/>
       <c r="O27" s="35"/>
       <c r="P27" s="35"/>
@@ -5653,10 +5926,10 @@
       <c r="G28" s="44"/>
       <c r="H28" s="35"/>
       <c r="I28" s="35"/>
-      <c r="J28" s="54"/>
-      <c r="K28" s="54"/>
-      <c r="L28" s="54"/>
-      <c r="M28" s="54"/>
+      <c r="J28" s="62"/>
+      <c r="K28" s="62"/>
+      <c r="L28" s="62"/>
+      <c r="M28" s="62"/>
       <c r="N28" s="35"/>
       <c r="O28" s="35"/>
       <c r="P28" s="35"/>
@@ -5812,7 +6085,7 @@
       <c r="D6" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="50" t="s">
         <v>359</v>
       </c>
     </row>
@@ -5939,17 +6212,17 @@
       <c r="E15" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G15" s="59" t="s">
+      <c r="G15" s="67" t="s">
         <v>335</v>
       </c>
-      <c r="H15" s="52"/>
-      <c r="I15" s="52"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="52"/>
-      <c r="L15" s="52"/>
-      <c r="M15" s="52"/>
-      <c r="N15" s="52"/>
-      <c r="O15" s="52"/>
+      <c r="H15" s="60"/>
+      <c r="I15" s="60"/>
+      <c r="J15" s="60"/>
+      <c r="K15" s="60"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="60"/>
+      <c r="N15" s="60"/>
+      <c r="O15" s="60"/>
     </row>
     <row r="16" spans="1:15">
       <c r="B16" s="35" t="s">
@@ -5964,15 +6237,15 @@
       <c r="E16" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="52"/>
-      <c r="N16" s="52"/>
-      <c r="O16" s="52"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="60"/>
+      <c r="L16" s="60"/>
+      <c r="M16" s="60"/>
+      <c r="N16" s="60"/>
+      <c r="O16" s="60"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="35" t="s">
@@ -5987,15 +6260,15 @@
       <c r="E17" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="52"/>
-      <c r="I17" s="52"/>
-      <c r="J17" s="52"/>
-      <c r="K17" s="52"/>
-      <c r="L17" s="52"/>
-      <c r="M17" s="52"/>
-      <c r="N17" s="52"/>
-      <c r="O17" s="52"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="60"/>
+      <c r="J17" s="60"/>
+      <c r="K17" s="60"/>
+      <c r="L17" s="60"/>
+      <c r="M17" s="60"/>
+      <c r="N17" s="60"/>
+      <c r="O17" s="60"/>
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="35" t="s">
@@ -6010,15 +6283,15 @@
       <c r="E18" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
-      <c r="I18" s="52"/>
-      <c r="J18" s="52"/>
-      <c r="K18" s="52"/>
-      <c r="L18" s="52"/>
-      <c r="M18" s="52"/>
-      <c r="N18" s="52"/>
-      <c r="O18" s="52"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="60"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="60"/>
+      <c r="K18" s="60"/>
+      <c r="L18" s="60"/>
+      <c r="M18" s="60"/>
+      <c r="N18" s="60"/>
+      <c r="O18" s="60"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="35" t="s">
@@ -6033,15 +6306,15 @@
       <c r="E19" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="52"/>
-      <c r="N19" s="52"/>
-      <c r="O19" s="52"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="60"/>
+      <c r="I19" s="60"/>
+      <c r="J19" s="60"/>
+      <c r="K19" s="60"/>
+      <c r="L19" s="60"/>
+      <c r="M19" s="60"/>
+      <c r="N19" s="60"/>
+      <c r="O19" s="60"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="35" t="s">
@@ -6056,15 +6329,15 @@
       <c r="E20" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="52"/>
-      <c r="J20" s="52"/>
-      <c r="K20" s="52"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="52"/>
-      <c r="N20" s="52"/>
-      <c r="O20" s="52"/>
+      <c r="G20" s="60"/>
+      <c r="H20" s="60"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="60"/>
+      <c r="K20" s="60"/>
+      <c r="L20" s="60"/>
+      <c r="M20" s="60"/>
+      <c r="N20" s="60"/>
+      <c r="O20" s="60"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="35" t="s">
@@ -6079,15 +6352,15 @@
       <c r="E21" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="52"/>
-      <c r="J21" s="52"/>
-      <c r="K21" s="52"/>
-      <c r="L21" s="52"/>
-      <c r="M21" s="52"/>
-      <c r="N21" s="52"/>
-      <c r="O21" s="52"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
+      <c r="I21" s="60"/>
+      <c r="J21" s="60"/>
+      <c r="K21" s="60"/>
+      <c r="L21" s="60"/>
+      <c r="M21" s="60"/>
+      <c r="N21" s="60"/>
+      <c r="O21" s="60"/>
     </row>
     <row r="22" spans="2:15">
       <c r="B22" s="35" t="s">
@@ -6102,15 +6375,15 @@
       <c r="E22" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="52"/>
-      <c r="K22" s="52"/>
-      <c r="L22" s="52"/>
-      <c r="M22" s="52"/>
-      <c r="N22" s="52"/>
-      <c r="O22" s="52"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="60"/>
+      <c r="K22" s="60"/>
+      <c r="L22" s="60"/>
+      <c r="M22" s="60"/>
+      <c r="N22" s="60"/>
+      <c r="O22" s="60"/>
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="35" t="s">
@@ -6125,15 +6398,15 @@
       <c r="E23" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="52"/>
-      <c r="N23" s="52"/>
-      <c r="O23" s="52"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
+      <c r="J23" s="60"/>
+      <c r="K23" s="60"/>
+      <c r="L23" s="60"/>
+      <c r="M23" s="60"/>
+      <c r="N23" s="60"/>
+      <c r="O23" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6184,13 +6457,13 @@
       <c r="E5" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="53" t="s">
+      <c r="G5" s="61" t="s">
         <v>347</v>
       </c>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="61"/>
     </row>
     <row r="6" spans="1:11" s="35" customFormat="1">
       <c r="B6" s="42" t="s">
@@ -6205,13 +6478,13 @@
       <c r="E6" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="52" t="s">
+      <c r="G6" s="60" t="s">
         <v>302</v>
       </c>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="52"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
     </row>
     <row r="7" spans="1:11" s="35" customFormat="1">
       <c r="B7" s="42" t="s">
@@ -6226,11 +6499,11 @@
       <c r="E7" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="60"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
     </row>
     <row r="8" spans="1:11" s="35" customFormat="1">
       <c r="B8" s="35" t="s">
@@ -6245,11 +6518,11 @@
       <c r="E8" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="60"/>
+      <c r="I8" s="60"/>
+      <c r="J8" s="60"/>
+      <c r="K8" s="60"/>
     </row>
     <row r="9" spans="1:11" s="35" customFormat="1">
       <c r="B9" s="35" t="s">
@@ -6264,11 +6537,11 @@
       <c r="E9" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="52"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="60"/>
+      <c r="I9" s="60"/>
+      <c r="J9" s="60"/>
+      <c r="K9" s="60"/>
     </row>
     <row r="10" spans="1:11" s="35" customFormat="1">
       <c r="B10" s="35" t="s">
@@ -6283,11 +6556,11 @@
       <c r="E10" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="52"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="60"/>
+      <c r="K10" s="60"/>
     </row>
     <row r="11" spans="1:11" s="35" customFormat="1"/>
     <row r="12" spans="1:11" s="35" customFormat="1">

</xml_diff>

<commit_message>
feat: Add applicant name and organization unit name fields to material requisition table
</commit_message>
<xml_diff>
--- a/aspnet-core/prototype/领用配送接口FS(2).xlsx
+++ b/aspnet-core/prototype/领用配送接口FS(2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\module-zero-core-template\aspnet-core\prototype\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A799F0-0386-42F9-891D-2C477C15FE55}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9432433-C3D0-48FA-9593-282C1DB7E931}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目录" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="397">
   <si>
     <t>A-LM-ABAP-WMZC588</t>
   </si>
@@ -1376,6 +1376,30 @@
   </si>
   <si>
     <t>13,3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>申请人描述</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>申请部门描述</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAME</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEPT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>60,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>40,0</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1648,7 +1672,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1792,6 +1816,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2458,7 +2485,7 @@
       <c r="E10" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G10" s="68" t="s">
+      <c r="G10" s="69" t="s">
         <v>309</v>
       </c>
       <c r="H10" s="2" t="s">
@@ -2478,7 +2505,7 @@
       <c r="E11" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="G11" s="57"/>
+      <c r="G11" s="58"/>
       <c r="H11" s="2" t="s">
         <v>154</v>
       </c>
@@ -2496,7 +2523,7 @@
       <c r="E12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="56"/>
+      <c r="G12" s="57"/>
       <c r="H12" s="2" t="s">
         <v>157</v>
       </c>
@@ -2514,7 +2541,7 @@
       <c r="E13" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="56"/>
+      <c r="G13" s="57"/>
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:8" s="15" customFormat="1">
@@ -2530,7 +2557,7 @@
       <c r="E14" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="57"/>
+      <c r="G14" s="58"/>
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1">
@@ -2833,25 +2860,25 @@
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="B36" s="70" t="s">
+      <c r="B36" s="71" t="s">
         <v>123</v>
       </c>
-      <c r="C36" s="69" t="s">
+      <c r="C36" s="70" t="s">
         <v>124</v>
       </c>
-      <c r="D36" s="69" t="s">
+      <c r="D36" s="70" t="s">
         <v>125</v>
       </c>
-      <c r="E36" s="68" t="s">
+      <c r="E36" s="69" t="s">
         <v>317</v>
       </c>
-      <c r="F36" s="57"/>
-      <c r="G36" s="56"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="57"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="B37" s="56"/>
-      <c r="C37" s="57"/>
-      <c r="D37" s="57"/>
+      <c r="B37" s="57"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
       <c r="E37" s="15" t="s">
         <v>126</v>
       </c>
@@ -3065,7 +3092,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="16.21875" style="14" customWidth="1"/>
@@ -3078,16 +3105,16 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="15" t="s">
@@ -3347,7 +3374,7 @@
       <c r="F23" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G23" s="58" t="s">
+      <c r="G23" s="59" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3367,7 +3394,7 @@
       <c r="F24" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G24" s="57"/>
+      <c r="G24" s="58"/>
     </row>
     <row r="25" spans="2:8">
       <c r="B25" s="15" t="s">
@@ -3385,7 +3412,7 @@
       <c r="F25" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G25" s="57"/>
+      <c r="G25" s="58"/>
     </row>
     <row r="26" spans="2:8">
       <c r="B26" s="15" t="s">
@@ -3403,7 +3430,7 @@
       <c r="F26" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G26" s="57"/>
+      <c r="G26" s="58"/>
     </row>
     <row r="27" spans="2:8" s="9" customFormat="1">
       <c r="B27" s="9" t="s">
@@ -3494,34 +3521,64 @@
       </c>
       <c r="H31" s="15"/>
     </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="15" t="s">
+    <row r="32" spans="2:8" s="55" customFormat="1">
+      <c r="B32" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D32" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="G32" s="8"/>
+    </row>
+    <row r="33" spans="1:7" s="55" customFormat="1">
+      <c r="B33" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="D33" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="G33" s="8"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B35" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C35" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D35" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
-      <c r="B34" s="15" t="s">
+    <row r="36" spans="1:7">
+      <c r="B36" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C36" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D36" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="E36" s="15" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3815,7 +3872,7 @@
       <c r="E22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="55" t="s">
+      <c r="F22" s="56" t="s">
         <v>153</v>
       </c>
     </row>
@@ -3832,7 +3889,7 @@
       <c r="E23" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="59"/>
+      <c r="F23" s="60"/>
     </row>
     <row r="24" spans="2:6" s="2" customFormat="1">
       <c r="B24" s="2" t="s">
@@ -3847,7 +3904,7 @@
       <c r="E24" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F24" s="59"/>
+      <c r="F24" s="60"/>
     </row>
     <row r="25" spans="2:6" s="2" customFormat="1">
       <c r="B25" s="2" t="s">
@@ -3862,7 +3919,7 @@
       <c r="E25" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="59"/>
+      <c r="F25" s="60"/>
     </row>
     <row r="26" spans="2:6" s="2" customFormat="1">
       <c r="B26" s="2" t="s">
@@ -3877,7 +3934,7 @@
       <c r="E26" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F26" s="59"/>
+      <c r="F26" s="60"/>
     </row>
     <row r="27" spans="2:6">
       <c r="B27" s="7" t="s">
@@ -3892,7 +3949,7 @@
       <c r="E27" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F27" s="56"/>
+      <c r="F27" s="57"/>
     </row>
     <row r="28" spans="2:6">
       <c r="B28" s="7" t="s">
@@ -3907,7 +3964,7 @@
       <c r="E28" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F28" s="56"/>
+      <c r="F28" s="57"/>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" s="15" t="s">
@@ -3922,7 +3979,7 @@
       <c r="E29" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="56"/>
+      <c r="F29" s="57"/>
     </row>
     <row r="30" spans="2:6">
       <c r="B30" s="15" t="s">
@@ -3937,7 +3994,7 @@
       <c r="E30" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="F30" s="56"/>
+      <c r="F30" s="57"/>
     </row>
     <row r="31" spans="2:6">
       <c r="B31" s="15" t="s">
@@ -3952,7 +4009,7 @@
       <c r="E31" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="56"/>
+      <c r="F31" s="57"/>
     </row>
     <row r="32" spans="2:6">
       <c r="F32" s="13"/>
@@ -4007,16 +4064,16 @@
       <c r="F36" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="G36" s="55" t="s">
+      <c r="G36" s="56" t="s">
         <v>184</v>
       </c>
-      <c r="H36" s="57"/>
-      <c r="I36" s="57"/>
-      <c r="J36" s="57"/>
-      <c r="K36" s="57"/>
-      <c r="L36" s="57"/>
-      <c r="M36" s="57"/>
-      <c r="N36" s="57"/>
+      <c r="H36" s="58"/>
+      <c r="I36" s="58"/>
+      <c r="J36" s="58"/>
+      <c r="K36" s="58"/>
+      <c r="L36" s="58"/>
+      <c r="M36" s="58"/>
+      <c r="N36" s="58"/>
     </row>
     <row r="37" spans="2:14">
       <c r="B37" s="15" t="s">
@@ -4031,16 +4088,16 @@
       <c r="E37" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="G37" s="55" t="s">
+      <c r="G37" s="56" t="s">
         <v>188</v>
       </c>
-      <c r="H37" s="57"/>
-      <c r="I37" s="57"/>
-      <c r="J37" s="57"/>
-      <c r="K37" s="57"/>
-      <c r="L37" s="57"/>
-      <c r="M37" s="57"/>
-      <c r="N37" s="57"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="58"/>
+      <c r="J37" s="58"/>
+      <c r="K37" s="58"/>
+      <c r="L37" s="58"/>
+      <c r="M37" s="58"/>
+      <c r="N37" s="58"/>
     </row>
     <row r="38" spans="2:14" s="34" customFormat="1">
       <c r="B38" s="7" t="s">
@@ -4082,132 +4139,132 @@
       </c>
     </row>
     <row r="42" spans="2:14">
-      <c r="B42" s="60" t="s">
+      <c r="B42" s="61" t="s">
         <v>190</v>
       </c>
-      <c r="C42" s="57"/>
-      <c r="D42" s="57"/>
-      <c r="E42" s="57"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="57"/>
-      <c r="H42" s="57"/>
-      <c r="I42" s="57"/>
-      <c r="J42" s="57"/>
-      <c r="K42" s="57"/>
-      <c r="L42" s="57"/>
-      <c r="M42" s="57"/>
+      <c r="C42" s="58"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="58"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="58"/>
+      <c r="K42" s="58"/>
+      <c r="L42" s="58"/>
+      <c r="M42" s="58"/>
     </row>
     <row r="43" spans="2:14">
-      <c r="B43" s="56"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="56"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="58"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="58"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="58"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="58"/>
+      <c r="L43" s="58"/>
+      <c r="M43" s="58"/>
     </row>
     <row r="44" spans="2:14">
-      <c r="B44" s="56"/>
-      <c r="C44" s="57"/>
-      <c r="D44" s="57"/>
-      <c r="E44" s="57"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="57"/>
-      <c r="H44" s="57"/>
-      <c r="I44" s="57"/>
-      <c r="J44" s="57"/>
-      <c r="K44" s="57"/>
-      <c r="L44" s="57"/>
-      <c r="M44" s="57"/>
+      <c r="B44" s="57"/>
+      <c r="C44" s="58"/>
+      <c r="D44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="57"/>
+      <c r="G44" s="58"/>
+      <c r="H44" s="58"/>
+      <c r="I44" s="58"/>
+      <c r="J44" s="58"/>
+      <c r="K44" s="58"/>
+      <c r="L44" s="58"/>
+      <c r="M44" s="58"/>
     </row>
     <row r="45" spans="2:14">
-      <c r="B45" s="56"/>
-      <c r="C45" s="57"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="57"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
-      <c r="I45" s="57"/>
-      <c r="J45" s="57"/>
-      <c r="K45" s="57"/>
-      <c r="L45" s="57"/>
-      <c r="M45" s="57"/>
+      <c r="B45" s="57"/>
+      <c r="C45" s="58"/>
+      <c r="D45" s="58"/>
+      <c r="E45" s="58"/>
+      <c r="F45" s="57"/>
+      <c r="G45" s="58"/>
+      <c r="H45" s="58"/>
+      <c r="I45" s="58"/>
+      <c r="J45" s="58"/>
+      <c r="K45" s="58"/>
+      <c r="L45" s="58"/>
+      <c r="M45" s="58"/>
     </row>
     <row r="46" spans="2:14">
-      <c r="B46" s="56"/>
-      <c r="C46" s="57"/>
-      <c r="D46" s="57"/>
-      <c r="E46" s="57"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="57"/>
-      <c r="H46" s="57"/>
-      <c r="I46" s="57"/>
-      <c r="J46" s="57"/>
-      <c r="K46" s="57"/>
-      <c r="L46" s="57"/>
-      <c r="M46" s="57"/>
+      <c r="B46" s="57"/>
+      <c r="C46" s="58"/>
+      <c r="D46" s="58"/>
+      <c r="E46" s="58"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="58"/>
+      <c r="H46" s="58"/>
+      <c r="I46" s="58"/>
+      <c r="J46" s="58"/>
+      <c r="K46" s="58"/>
+      <c r="L46" s="58"/>
+      <c r="M46" s="58"/>
     </row>
     <row r="47" spans="2:14">
-      <c r="B47" s="56"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="56"/>
-      <c r="G47" s="57"/>
-      <c r="H47" s="57"/>
-      <c r="I47" s="57"/>
-      <c r="J47" s="57"/>
-      <c r="K47" s="57"/>
-      <c r="L47" s="57"/>
-      <c r="M47" s="57"/>
+      <c r="B47" s="57"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="57"/>
+      <c r="G47" s="58"/>
+      <c r="H47" s="58"/>
+      <c r="I47" s="58"/>
+      <c r="J47" s="58"/>
+      <c r="K47" s="58"/>
+      <c r="L47" s="58"/>
+      <c r="M47" s="58"/>
     </row>
     <row r="48" spans="2:14">
-      <c r="B48" s="56"/>
-      <c r="C48" s="57"/>
-      <c r="D48" s="57"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="57"/>
-      <c r="H48" s="57"/>
-      <c r="I48" s="57"/>
-      <c r="J48" s="57"/>
-      <c r="K48" s="57"/>
-      <c r="L48" s="57"/>
-      <c r="M48" s="57"/>
+      <c r="B48" s="57"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="57"/>
+      <c r="G48" s="58"/>
+      <c r="H48" s="58"/>
+      <c r="I48" s="58"/>
+      <c r="J48" s="58"/>
+      <c r="K48" s="58"/>
+      <c r="L48" s="58"/>
+      <c r="M48" s="58"/>
     </row>
     <row r="49" spans="2:13">
-      <c r="B49" s="56"/>
-      <c r="C49" s="57"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="57"/>
-      <c r="H49" s="57"/>
-      <c r="I49" s="57"/>
-      <c r="J49" s="57"/>
-      <c r="K49" s="57"/>
-      <c r="L49" s="57"/>
-      <c r="M49" s="57"/>
+      <c r="B49" s="57"/>
+      <c r="C49" s="58"/>
+      <c r="D49" s="58"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="57"/>
+      <c r="G49" s="58"/>
+      <c r="H49" s="58"/>
+      <c r="I49" s="58"/>
+      <c r="J49" s="58"/>
+      <c r="K49" s="58"/>
+      <c r="L49" s="58"/>
+      <c r="M49" s="58"/>
     </row>
     <row r="50" spans="2:13">
-      <c r="B50" s="56"/>
-      <c r="C50" s="57"/>
-      <c r="D50" s="57"/>
-      <c r="E50" s="57"/>
-      <c r="F50" s="56"/>
-      <c r="G50" s="57"/>
-      <c r="H50" s="57"/>
-      <c r="I50" s="57"/>
-      <c r="J50" s="57"/>
-      <c r="K50" s="57"/>
-      <c r="L50" s="57"/>
-      <c r="M50" s="57"/>
+      <c r="B50" s="57"/>
+      <c r="C50" s="58"/>
+      <c r="D50" s="58"/>
+      <c r="E50" s="58"/>
+      <c r="F50" s="57"/>
+      <c r="G50" s="58"/>
+      <c r="H50" s="58"/>
+      <c r="I50" s="58"/>
+      <c r="J50" s="58"/>
+      <c r="K50" s="58"/>
+      <c r="L50" s="58"/>
+      <c r="M50" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -5294,13 +5351,13 @@
       <c r="E4" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="61" t="s">
+      <c r="F4" s="62" t="s">
         <v>347</v>
       </c>
-      <c r="G4" s="61"/>
-      <c r="H4" s="61"/>
-      <c r="I4" s="61"/>
-      <c r="J4" s="61"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
       <c r="K4" s="35"/>
       <c r="L4" s="35"/>
       <c r="M4" s="35"/>
@@ -5599,14 +5656,14 @@
       <c r="G15" s="35"/>
       <c r="H15" s="35"/>
       <c r="I15" s="35"/>
-      <c r="J15" s="60" t="s">
+      <c r="J15" s="61" t="s">
         <v>295</v>
       </c>
-      <c r="K15" s="66"/>
-      <c r="L15" s="66"/>
-      <c r="M15" s="66"/>
-      <c r="N15" s="66"/>
-      <c r="O15" s="66"/>
+      <c r="K15" s="67"/>
+      <c r="L15" s="67"/>
+      <c r="M15" s="67"/>
+      <c r="N15" s="67"/>
+      <c r="O15" s="67"/>
       <c r="P15" s="35"/>
       <c r="Q15" s="35"/>
     </row>
@@ -5628,12 +5685,12 @@
       <c r="G16" s="35"/>
       <c r="H16" s="35"/>
       <c r="I16" s="35"/>
-      <c r="J16" s="66"/>
-      <c r="K16" s="66"/>
-      <c r="L16" s="66"/>
-      <c r="M16" s="66"/>
-      <c r="N16" s="66"/>
-      <c r="O16" s="66"/>
+      <c r="J16" s="67"/>
+      <c r="K16" s="67"/>
+      <c r="L16" s="67"/>
+      <c r="M16" s="67"/>
+      <c r="N16" s="67"/>
+      <c r="O16" s="67"/>
       <c r="P16" s="35"/>
       <c r="Q16" s="35"/>
     </row>
@@ -5655,12 +5712,12 @@
       <c r="G17" s="35"/>
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="66"/>
-      <c r="L17" s="66"/>
-      <c r="M17" s="66"/>
-      <c r="N17" s="66"/>
-      <c r="O17" s="66"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="67"/>
+      <c r="L17" s="67"/>
+      <c r="M17" s="67"/>
+      <c r="N17" s="67"/>
+      <c r="O17" s="67"/>
       <c r="P17" s="35"/>
       <c r="Q17" s="35"/>
     </row>
@@ -5682,12 +5739,12 @@
       <c r="G18" s="35"/>
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
-      <c r="J18" s="66"/>
-      <c r="K18" s="66"/>
-      <c r="L18" s="66"/>
-      <c r="M18" s="66"/>
-      <c r="N18" s="66"/>
-      <c r="O18" s="66"/>
+      <c r="J18" s="67"/>
+      <c r="K18" s="67"/>
+      <c r="L18" s="67"/>
+      <c r="M18" s="67"/>
+      <c r="N18" s="67"/>
+      <c r="O18" s="67"/>
       <c r="P18" s="35"/>
       <c r="Q18" s="35"/>
     </row>
@@ -5701,12 +5758,12 @@
       <c r="G19" s="35"/>
       <c r="H19" s="35"/>
       <c r="I19" s="35"/>
-      <c r="J19" s="66"/>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
-      <c r="M19" s="66"/>
-      <c r="N19" s="66"/>
-      <c r="O19" s="66"/>
+      <c r="J19" s="67"/>
+      <c r="K19" s="67"/>
+      <c r="L19" s="67"/>
+      <c r="M19" s="67"/>
+      <c r="N19" s="67"/>
+      <c r="O19" s="67"/>
       <c r="P19" s="35"/>
       <c r="Q19" s="35"/>
     </row>
@@ -5720,12 +5777,12 @@
       <c r="G20" s="35"/>
       <c r="H20" s="35"/>
       <c r="I20" s="35"/>
-      <c r="J20" s="66"/>
-      <c r="K20" s="66"/>
-      <c r="L20" s="66"/>
-      <c r="M20" s="66"/>
-      <c r="N20" s="66"/>
-      <c r="O20" s="66"/>
+      <c r="J20" s="67"/>
+      <c r="K20" s="67"/>
+      <c r="L20" s="67"/>
+      <c r="M20" s="67"/>
+      <c r="N20" s="67"/>
+      <c r="O20" s="67"/>
       <c r="P20" s="35"/>
       <c r="Q20" s="35"/>
     </row>
@@ -5739,12 +5796,12 @@
       <c r="G21" s="35"/>
       <c r="H21" s="35"/>
       <c r="I21" s="35"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
-      <c r="M21" s="66"/>
-      <c r="N21" s="66"/>
-      <c r="O21" s="66"/>
+      <c r="J21" s="67"/>
+      <c r="K21" s="67"/>
+      <c r="L21" s="67"/>
+      <c r="M21" s="67"/>
+      <c r="N21" s="67"/>
+      <c r="O21" s="67"/>
       <c r="P21" s="35"/>
       <c r="Q21" s="35"/>
     </row>
@@ -5768,47 +5825,47 @@
       <c r="G22" s="35"/>
       <c r="H22" s="35"/>
       <c r="I22" s="35"/>
-      <c r="J22" s="66"/>
-      <c r="K22" s="66"/>
-      <c r="L22" s="66"/>
-      <c r="M22" s="66"/>
-      <c r="N22" s="66"/>
-      <c r="O22" s="66"/>
+      <c r="J22" s="67"/>
+      <c r="K22" s="67"/>
+      <c r="L22" s="67"/>
+      <c r="M22" s="67"/>
+      <c r="N22" s="67"/>
+      <c r="O22" s="67"/>
       <c r="P22" s="35"/>
       <c r="Q22" s="35"/>
     </row>
     <row r="23" spans="1:17" ht="34.950000000000003" customHeight="1">
       <c r="A23" s="35"/>
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="64" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="64" t="s">
+      <c r="C23" s="65" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="64" t="s">
+      <c r="D23" s="65" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="65" t="s">
+      <c r="E23" s="66" t="s">
         <v>348</v>
       </c>
-      <c r="F23" s="65"/>
-      <c r="G23" s="65"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="66"/>
       <c r="H23" s="35"/>
       <c r="I23" s="35"/>
-      <c r="J23" s="66"/>
-      <c r="K23" s="66"/>
-      <c r="L23" s="66"/>
-      <c r="M23" s="66"/>
-      <c r="N23" s="66"/>
-      <c r="O23" s="66"/>
+      <c r="J23" s="67"/>
+      <c r="K23" s="67"/>
+      <c r="L23" s="67"/>
+      <c r="M23" s="67"/>
+      <c r="N23" s="67"/>
+      <c r="O23" s="67"/>
       <c r="P23" s="35"/>
       <c r="Q23" s="35"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="35"/>
-      <c r="B24" s="63"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="65"/>
+      <c r="D24" s="65"/>
       <c r="E24" s="43" t="s">
         <v>126</v>
       </c>
@@ -5816,12 +5873,12 @@
       <c r="G24" s="44"/>
       <c r="H24" s="35"/>
       <c r="I24" s="35"/>
-      <c r="J24" s="66"/>
-      <c r="K24" s="66"/>
-      <c r="L24" s="66"/>
-      <c r="M24" s="66"/>
-      <c r="N24" s="66"/>
-      <c r="O24" s="66"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
+      <c r="L24" s="67"/>
+      <c r="M24" s="67"/>
+      <c r="N24" s="67"/>
+      <c r="O24" s="67"/>
       <c r="P24" s="35"/>
       <c r="Q24" s="35"/>
     </row>
@@ -5870,12 +5927,12 @@
       <c r="G26" s="44"/>
       <c r="H26" s="35"/>
       <c r="I26" s="35"/>
-      <c r="J26" s="62" t="s">
+      <c r="J26" s="63" t="s">
         <v>349</v>
       </c>
-      <c r="K26" s="62"/>
-      <c r="L26" s="62"/>
-      <c r="M26" s="62"/>
+      <c r="K26" s="63"/>
+      <c r="L26" s="63"/>
+      <c r="M26" s="63"/>
       <c r="N26" s="35"/>
       <c r="O26" s="35"/>
       <c r="P26" s="35"/>
@@ -5899,10 +5956,10 @@
       <c r="G27" s="44"/>
       <c r="H27" s="35"/>
       <c r="I27" s="35"/>
-      <c r="J27" s="62"/>
-      <c r="K27" s="62"/>
-      <c r="L27" s="62"/>
-      <c r="M27" s="62"/>
+      <c r="J27" s="63"/>
+      <c r="K27" s="63"/>
+      <c r="L27" s="63"/>
+      <c r="M27" s="63"/>
       <c r="N27" s="35"/>
       <c r="O27" s="35"/>
       <c r="P27" s="35"/>
@@ -5926,10 +5983,10 @@
       <c r="G28" s="44"/>
       <c r="H28" s="35"/>
       <c r="I28" s="35"/>
-      <c r="J28" s="62"/>
-      <c r="K28" s="62"/>
-      <c r="L28" s="62"/>
-      <c r="M28" s="62"/>
+      <c r="J28" s="63"/>
+      <c r="K28" s="63"/>
+      <c r="L28" s="63"/>
+      <c r="M28" s="63"/>
       <c r="N28" s="35"/>
       <c r="O28" s="35"/>
       <c r="P28" s="35"/>
@@ -6212,17 +6269,17 @@
       <c r="E15" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G15" s="67" t="s">
+      <c r="G15" s="68" t="s">
         <v>335</v>
       </c>
-      <c r="H15" s="60"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60"/>
+      <c r="H15" s="61"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="61"/>
+      <c r="L15" s="61"/>
+      <c r="M15" s="61"/>
+      <c r="N15" s="61"/>
+      <c r="O15" s="61"/>
     </row>
     <row r="16" spans="1:15">
       <c r="B16" s="35" t="s">
@@ -6237,15 +6294,15 @@
       <c r="E16" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="60"/>
-      <c r="M16" s="60"/>
-      <c r="N16" s="60"/>
-      <c r="O16" s="60"/>
+      <c r="G16" s="61"/>
+      <c r="H16" s="61"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61"/>
+      <c r="N16" s="61"/>
+      <c r="O16" s="61"/>
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="35" t="s">
@@ -6260,15 +6317,15 @@
       <c r="E17" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="60"/>
-      <c r="L17" s="60"/>
-      <c r="M17" s="60"/>
-      <c r="N17" s="60"/>
-      <c r="O17" s="60"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="61"/>
+      <c r="N17" s="61"/>
+      <c r="O17" s="61"/>
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="35" t="s">
@@ -6283,15 +6340,15 @@
       <c r="E18" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G18" s="60"/>
-      <c r="H18" s="60"/>
-      <c r="I18" s="60"/>
-      <c r="J18" s="60"/>
-      <c r="K18" s="60"/>
-      <c r="L18" s="60"/>
-      <c r="M18" s="60"/>
-      <c r="N18" s="60"/>
-      <c r="O18" s="60"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="61"/>
+      <c r="K18" s="61"/>
+      <c r="L18" s="61"/>
+      <c r="M18" s="61"/>
+      <c r="N18" s="61"/>
+      <c r="O18" s="61"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="35" t="s">
@@ -6306,15 +6363,15 @@
       <c r="E19" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="60"/>
-      <c r="H19" s="60"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="60"/>
-      <c r="L19" s="60"/>
-      <c r="M19" s="60"/>
-      <c r="N19" s="60"/>
-      <c r="O19" s="60"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="61"/>
+      <c r="J19" s="61"/>
+      <c r="K19" s="61"/>
+      <c r="L19" s="61"/>
+      <c r="M19" s="61"/>
+      <c r="N19" s="61"/>
+      <c r="O19" s="61"/>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="35" t="s">
@@ -6329,15 +6386,15 @@
       <c r="E20" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="60"/>
-      <c r="M20" s="60"/>
-      <c r="N20" s="60"/>
-      <c r="O20" s="60"/>
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="61"/>
+      <c r="J20" s="61"/>
+      <c r="K20" s="61"/>
+      <c r="L20" s="61"/>
+      <c r="M20" s="61"/>
+      <c r="N20" s="61"/>
+      <c r="O20" s="61"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="35" t="s">
@@ -6352,15 +6409,15 @@
       <c r="E21" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="60"/>
-      <c r="K21" s="60"/>
-      <c r="L21" s="60"/>
-      <c r="M21" s="60"/>
-      <c r="N21" s="60"/>
-      <c r="O21" s="60"/>
+      <c r="G21" s="61"/>
+      <c r="H21" s="61"/>
+      <c r="I21" s="61"/>
+      <c r="J21" s="61"/>
+      <c r="K21" s="61"/>
+      <c r="L21" s="61"/>
+      <c r="M21" s="61"/>
+      <c r="N21" s="61"/>
+      <c r="O21" s="61"/>
     </row>
     <row r="22" spans="2:15">
       <c r="B22" s="35" t="s">
@@ -6375,15 +6432,15 @@
       <c r="E22" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="60"/>
-      <c r="M22" s="60"/>
-      <c r="N22" s="60"/>
-      <c r="O22" s="60"/>
+      <c r="G22" s="61"/>
+      <c r="H22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="61"/>
+      <c r="L22" s="61"/>
+      <c r="M22" s="61"/>
+      <c r="N22" s="61"/>
+      <c r="O22" s="61"/>
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="35" t="s">
@@ -6398,15 +6455,15 @@
       <c r="E23" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="60"/>
-      <c r="K23" s="60"/>
-      <c r="L23" s="60"/>
-      <c r="M23" s="60"/>
-      <c r="N23" s="60"/>
-      <c r="O23" s="60"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="61"/>
+      <c r="L23" s="61"/>
+      <c r="M23" s="61"/>
+      <c r="N23" s="61"/>
+      <c r="O23" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6457,13 +6514,13 @@
       <c r="E5" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="62" t="s">
         <v>347</v>
       </c>
-      <c r="H5" s="61"/>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="61"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
     </row>
     <row r="6" spans="1:11" s="35" customFormat="1">
       <c r="B6" s="42" t="s">
@@ -6478,13 +6535,13 @@
       <c r="E6" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="61" t="s">
         <v>302</v>
       </c>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
+      <c r="H6" s="61"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="61"/>
     </row>
     <row r="7" spans="1:11" s="35" customFormat="1">
       <c r="B7" s="42" t="s">
@@ -6499,11 +6556,11 @@
       <c r="E7" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="60"/>
-      <c r="K7" s="60"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="61"/>
+      <c r="I7" s="61"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="61"/>
     </row>
     <row r="8" spans="1:11" s="35" customFormat="1">
       <c r="B8" s="35" t="s">
@@ -6518,11 +6575,11 @@
       <c r="E8" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="60"/>
-      <c r="K8" s="60"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="61"/>
+      <c r="K8" s="61"/>
     </row>
     <row r="9" spans="1:11" s="35" customFormat="1">
       <c r="B9" s="35" t="s">
@@ -6537,11 +6594,11 @@
       <c r="E9" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
-      <c r="I9" s="60"/>
-      <c r="J9" s="60"/>
-      <c r="K9" s="60"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
     </row>
     <row r="10" spans="1:11" s="35" customFormat="1">
       <c r="B10" s="35" t="s">
@@ -6556,11 +6613,11 @@
       <c r="E10" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
-      <c r="K10" s="60"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
+      <c r="K10" s="61"/>
     </row>
     <row r="11" spans="1:11" s="35" customFormat="1"/>
     <row r="12" spans="1:11" s="35" customFormat="1">

</xml_diff>